<commit_message>
QC summary: add FRiP/TSS/gene-body metrics and comparison with Chen et al.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118hMfJWJZ4DaiswK3vUJeT
</commit_message>
<xml_diff>
--- a/cfEpi_20261026_QC_summary.xlsx
+++ b/cfEpi_20261026_QC_summary.xlsx
@@ -11,9 +11,10 @@
     <sheet name="Per_library" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="By_mark" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="By_batch" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="vs_Chen2026" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Per_library!$A$4:$R$28</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Per_library!$A$4:$U$28</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="131">
   <si>
     <t xml:space="preserve">cf-EpiTracing run 20261026 — QC summary per library</t>
   </si>
@@ -81,6 +82,15 @@
     <t xml:space="preserve">GC % (aligned)</t>
   </si>
   <si>
+    <t xml:space="preserve">FRiP %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% reads at TSS ±1 kb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% reads in gene bodies</t>
+  </si>
+  <si>
     <t xml:space="preserve">Verdict</t>
   </si>
   <si>
@@ -216,7 +226,7 @@
     <t xml:space="preserve">Caution</t>
   </si>
   <si>
-    <t xml:space="preserve">Borderline (target &gt;2); r=0.78 with cfEpi_12</t>
+    <t xml:space="preserve">Gene-body enrichment confirmed in log2(H3K36me3/IgG) profile; weaker than cfEpi_12; r=0.78 with cfEpi_12</t>
   </si>
   <si>
     <t xml:space="preserve">cfEpi_18</t>
@@ -243,7 +253,7 @@
     <t xml:space="preserve">cfEpi_22</t>
   </si>
   <si>
-    <t xml:space="preserve">Borderline (target &gt;2); r=0.74–0.77 with cfEpi_12/17</t>
+    <t xml:space="preserve">Gene-body enrichment confirmed in log2(H3K36me3/IgG) profile; weakest donor; r=0.74–0.77 with cfEpi_12/17</t>
   </si>
   <si>
     <t xml:space="preserve">cfEpi_23</t>
@@ -279,6 +289,15 @@
     <t xml:space="preserve">Overall assessment</t>
   </si>
   <si>
+    <t xml:space="preserve">Mean FRiP %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean % reads at TSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean % reads in gene bodies</t>
+  </si>
+  <si>
     <t xml:space="preserve">Most robust: strong in all 3 donors; use as positive control every run</t>
   </si>
   <si>
@@ -328,6 +347,78 @@
   </si>
   <si>
     <t xml:space="preserve">Strongest H3K4me3; H3K36me3 near-pass in both donors; HC9 high dm6; IgG cfEpi_24 contaminated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparison with Chen et al., Nature 2026 (Extended Data figure: cf-EpiTracing vs cfChIP by plasma volume)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chen et al. values read from the published figure (small print; approximate). "Reads" as labelled in the figure. This study: 200 µl plasma, usable libraries; reads = unique human reads after filtering (2 × unique fragments). DOI 10.1038/s41586-026-10224-0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plasma volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reads (M)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peaks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chen et al. cf-EpiTracing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25 µl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 µl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 µl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 µl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">500 µl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,000 µl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chen et al. cfChIP (Sadeh et al.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_7 (HC1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_10 (HC1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_15 (HC8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_20 (HC9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_1 (HC1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_4 (HC1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_8 (HC1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_11 (HC1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_16 (HC8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This study cfEpi_21 (HC9)</t>
   </si>
 </sst>
 </file>
@@ -400,7 +491,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -416,7 +507,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -428,6 +519,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
         <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
@@ -481,7 +578,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -535,6 +632,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -617,7 +730,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -843,7 +956,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -855,9 +968,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="9" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="13" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -925,19 +1039,28 @@
       <c r="R4" s="3" t="s">
         <v>19</v>
       </c>
+      <c r="S4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>58251150</v>
@@ -975,25 +1098,34 @@
       <c r="P5" s="6" t="n">
         <v>52.1</v>
       </c>
-      <c r="Q5" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R5" s="4" t="s">
-        <v>25</v>
+      <c r="Q5" s="6" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="T5" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>33995549</v>
@@ -1031,25 +1163,34 @@
       <c r="P6" s="6" t="n">
         <v>47.7</v>
       </c>
-      <c r="Q6" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="R6" s="4" t="s">
-        <v>29</v>
+      <c r="Q6" s="6" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="T6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U6" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>14717342</v>
@@ -1087,25 +1228,34 @@
       <c r="P7" s="6" t="n">
         <v>46.4</v>
       </c>
-      <c r="Q7" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R7" s="4" t="s">
-        <v>32</v>
+      <c r="Q7" s="6" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="T7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>21471046</v>
@@ -1143,25 +1293,34 @@
       <c r="P8" s="6" t="n">
         <v>50.5</v>
       </c>
-      <c r="Q8" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R8" s="4" t="s">
-        <v>35</v>
+      <c r="Q8" s="6" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S8" s="6" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="T8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>8104510</v>
@@ -1199,25 +1358,34 @@
       <c r="P9" s="6" t="n">
         <v>45.1</v>
       </c>
-      <c r="Q9" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="R9" s="4" t="s">
-        <v>37</v>
+      <c r="Q9" s="6" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="S9" s="6" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="T9" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U9" s="4" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>16656297</v>
@@ -1255,25 +1423,34 @@
       <c r="P10" s="6" t="n">
         <v>48.9</v>
       </c>
-      <c r="Q10" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R10" s="4" t="s">
-        <v>39</v>
+      <c r="Q10" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="S10" s="6" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="T10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U10" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>8488580</v>
@@ -1311,23 +1488,32 @@
       <c r="P11" s="6" t="n">
         <v>50.4</v>
       </c>
-      <c r="Q11" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R11" s="4"/>
+      <c r="Q11" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="T11" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>7225322</v>
@@ -1365,23 +1551,32 @@
       <c r="P12" s="6" t="n">
         <v>47.2</v>
       </c>
-      <c r="Q12" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R12" s="4"/>
+      <c r="Q12" s="6" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="S12" s="6" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="T12" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>5114468</v>
@@ -1419,25 +1614,34 @@
       <c r="P13" s="6" t="n">
         <v>47.1</v>
       </c>
-      <c r="Q13" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R13" s="4" t="s">
-        <v>45</v>
+      <c r="Q13" s="6" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="T13" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U13" s="4" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>4073425</v>
@@ -1467,7 +1671,7 @@
         <v>1.22</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="O14" s="5" t="n">
         <v>18787</v>
@@ -1475,25 +1679,34 @@
       <c r="P14" s="6" t="n">
         <v>53.5</v>
       </c>
-      <c r="Q14" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R14" s="4" t="s">
-        <v>48</v>
+      <c r="Q14" s="6" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="S14" s="6" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="T14" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U14" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>5226253</v>
@@ -1531,25 +1744,34 @@
       <c r="P15" s="6" t="n">
         <v>49.6</v>
       </c>
-      <c r="Q15" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R15" s="4" t="s">
-        <v>50</v>
+      <c r="Q15" s="6" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="T15" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U15" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>37008528</v>
@@ -1587,25 +1809,34 @@
       <c r="P16" s="6" t="n">
         <v>52.1</v>
       </c>
-      <c r="Q16" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R16" s="4" t="s">
-        <v>52</v>
+      <c r="Q16" s="6" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="R16" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S16" s="6" t="n">
+        <v>66.9</v>
+      </c>
+      <c r="T16" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U16" s="4" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E17" s="5" t="n">
         <v>3431114</v>
@@ -1643,23 +1874,32 @@
       <c r="P17" s="6" t="n">
         <v>47.7</v>
       </c>
-      <c r="Q17" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R17" s="4"/>
+      <c r="Q17" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="R17" s="6" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="S17" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="T17" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>8603181</v>
@@ -1697,25 +1937,34 @@
       <c r="P18" s="6" t="n">
         <v>43.6</v>
       </c>
-      <c r="Q18" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R18" s="4" t="s">
-        <v>55</v>
+      <c r="Q18" s="6" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R18" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="S18" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="T18" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U18" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E19" s="5" t="n">
         <v>7132357</v>
@@ -1753,25 +2002,34 @@
       <c r="P19" s="6" t="n">
         <v>52.7</v>
       </c>
-      <c r="Q19" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R19" s="4" t="s">
-        <v>58</v>
+      <c r="Q19" s="6" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="S19" s="6" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="T19" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U19" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E20" s="5" t="n">
         <v>7532211</v>
@@ -1809,25 +2067,34 @@
       <c r="P20" s="6" t="n">
         <v>47.8</v>
       </c>
-      <c r="Q20" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R20" s="4" t="s">
-        <v>60</v>
+      <c r="Q20" s="6" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="R20" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S20" s="6" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="T20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U20" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E21" s="5" t="n">
         <v>13677919</v>
@@ -1865,25 +2132,34 @@
       <c r="P21" s="6" t="n">
         <v>52.9</v>
       </c>
-      <c r="Q21" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="R21" s="4" t="s">
-        <v>63</v>
+      <c r="Q21" s="6" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="R21" s="6" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="S21" s="6" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="T21" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="U21" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>8359901</v>
@@ -1921,25 +2197,34 @@
       <c r="P22" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="Q22" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R22" s="4" t="s">
-        <v>60</v>
+      <c r="Q22" s="6" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="R22" s="6" t="n">
+        <v>8.3</v>
+      </c>
+      <c r="S22" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="T22" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U22" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E23" s="5" t="n">
         <v>7875800</v>
@@ -1977,25 +2262,34 @@
       <c r="P23" s="6" t="n">
         <v>47.4</v>
       </c>
-      <c r="Q23" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R23" s="4" t="s">
-        <v>39</v>
+      <c r="Q23" s="6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="R23" s="6" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="S23" s="6" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="T23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U23" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>8371828</v>
@@ -2033,25 +2327,34 @@
       <c r="P24" s="6" t="n">
         <v>51.4</v>
       </c>
-      <c r="Q24" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R24" s="4" t="s">
-        <v>68</v>
+      <c r="Q24" s="6" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="R24" s="6" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="S24" s="6" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="T24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U24" s="4" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E25" s="5" t="n">
         <v>7716460</v>
@@ -2089,25 +2392,34 @@
       <c r="P25" s="6" t="n">
         <v>47.8</v>
       </c>
-      <c r="Q25" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R25" s="4" t="s">
-        <v>70</v>
+      <c r="Q25" s="6" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="R25" s="6" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="S25" s="6" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="T25" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U25" s="4" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E26" s="5" t="n">
         <v>11179542</v>
@@ -2145,25 +2457,34 @@
       <c r="P26" s="6" t="n">
         <v>50.4</v>
       </c>
-      <c r="Q26" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="R26" s="4" t="s">
-        <v>72</v>
+      <c r="Q26" s="6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="R26" s="6" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="S26" s="6" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="T26" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="U26" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E27" s="5" t="n">
         <v>7055235</v>
@@ -2201,25 +2522,34 @@
       <c r="P27" s="6" t="n">
         <v>47.4</v>
       </c>
-      <c r="Q27" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="R27" s="4" t="s">
-        <v>70</v>
+      <c r="Q27" s="6" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="S27" s="6" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="T27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U27" s="4" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E28" s="5" t="n">
         <v>6074464</v>
@@ -2257,15 +2587,24 @@
       <c r="P28" s="6" t="n">
         <v>46.1</v>
       </c>
-      <c r="Q28" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="R28" s="4" t="s">
-        <v>75</v>
+      <c r="Q28" s="6" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="R28" s="6" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="S28" s="6" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="T28" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U28" s="4" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:R28"/>
+  <autoFilter ref="A4:U28"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2282,7 +2621,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -2293,197 +2632,268 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>83</v>
+        <v>86</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B4" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A4,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>4</v>
       </c>
       <c r="C4" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A4,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>14.405</v>
       </c>
       <c r="D4" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A4,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>1.1</v>
       </c>
       <c r="E4" s="5" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A4,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>1079330.25</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A4,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>70.25</v>
       </c>
       <c r="G4" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A4,Per_library!$Q$5:$Q$28,"Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"Exclude")</f>
         <v>0</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>84</v>
+        <v>90</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$Q$5:$Q$28,Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>39.55</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$R$5:$R$28,Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>30.1</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$S$5:$S$28,Per_library!$D$5:$D$28,A4,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>60.025</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B5" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A5,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>6</v>
       </c>
       <c r="C5" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A5,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>4.44833333333333</v>
       </c>
       <c r="D5" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A5,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>1.355</v>
       </c>
       <c r="E5" s="5" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A5,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>1060799.16666667</v>
       </c>
       <c r="F5" s="6" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A5,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>79.5666666666667</v>
       </c>
       <c r="G5" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A5,Per_library!$Q$5:$Q$28,"Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"Exclude")</f>
         <v>0</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>85</v>
+        <v>91</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$Q$5:$Q$28,Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>23.5666666666667</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$R$5:$R$28,Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>12.2333333333333</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$S$5:$S$28,Per_library!$D$5:$D$28,A5,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>56.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B6" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A6,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>4</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A6,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>4.095</v>
       </c>
       <c r="D6" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A6,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>1.0375</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A6,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>636766</v>
       </c>
       <c r="F6" s="6" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A6,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>74.6</v>
       </c>
       <c r="G6" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A6,Per_library!$Q$5:$Q$28,"Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"Exclude")</f>
         <v>0</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>86</v>
+        <v>92</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$Q$5:$Q$28,Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>14.225</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$R$5:$R$28,Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>14.05</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$S$5:$S$28,Per_library!$D$5:$D$28,A6,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>54.275</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B7" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A7,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>3</v>
       </c>
       <c r="C7" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A7,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>1.02333333333333</v>
       </c>
       <c r="D7" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A7,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>1.97333333333333</v>
       </c>
       <c r="E7" s="5" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A7,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>3856970.33333333</v>
       </c>
       <c r="F7" s="6" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A7,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>65.2</v>
       </c>
       <c r="G7" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A7,Per_library!$Q$5:$Q$28,"Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"Exclude")</f>
         <v>2</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>87</v>
+        <v>93</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$Q$5:$Q$28,Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>12.5666666666667</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$R$5:$R$28,Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>5.33333333333333</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$S$5:$S$28,Per_library!$D$5:$D$28,A7,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>62.4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B8" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A8,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>4</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A8,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$J$5:$J$28,Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>1.39</v>
       </c>
       <c r="D8" s="8" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A8,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$M$5:$M$28,Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>0.99</v>
       </c>
       <c r="E8" s="5" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A8,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$H$5:$H$28,Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>924642</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A8,Per_library!$Q$5:$Q$28,"&lt;&gt;Exclude")</f>
+        <f aca="false">AVERAGEIFS(Per_library!$G$5:$G$28,Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
         <v>73</v>
       </c>
       <c r="G8" s="4" t="n">
-        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A8,Per_library!$Q$5:$Q$28,"Exclude")</f>
+        <f aca="false">COUNTIFS(Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"Exclude")</f>
         <v>1</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$Q$5:$Q$28,Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>4.325</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$R$5:$R$28,Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>2.8</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <f aca="false">AVERAGEIFS(Per_library!$S$5:$S$28,Per_library!$D$5:$D$28,A8,Per_library!$T$5:$T$28,"&lt;&gt;Exclude")</f>
+        <v>49.275</v>
       </c>
     </row>
   </sheetData>
@@ -2515,35 +2925,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B4" s="4" t="n">
         <f aca="false">COUNTA(Per_library!A5:A10)</f>
@@ -2566,12 +2976,12 @@
         <v>0.0118333333333333</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">COUNTA(Per_library!A11:A18)</f>
@@ -2594,12 +3004,12 @@
         <v>0.017375</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">COUNTA(Per_library!A19:A28)</f>
@@ -2622,7 +3032,624 @@
         <v>0.0915</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>100</v>
+        <v>106</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>13646</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>35295</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>20603</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>30292</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>71.1</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>33706</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>29975</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>5478</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>5082</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>17170</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>10587</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>18787</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>13356</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>22058</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>16243</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>21460</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>23642</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>32289</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>68.9</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>32907</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>45296</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>10551</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>8763</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>20531</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>60132</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="F28" s="17" t="n">
+        <v>40608</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="F29" s="17" t="n">
+        <v>17285</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <v>51942</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="F31" s="17" t="n">
+        <v>7834</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="F32" s="17" t="n">
+        <v>587</v>
       </c>
     </row>
   </sheetData>

</xml_diff>